<commit_message>
WIP: add time registration call
</commit_message>
<xml_diff>
--- a/data/timeregistrations.xlsx
+++ b/data/timeregistrations.xlsx
@@ -5,10 +5,11 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="employees" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="log" sheetId="2" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -20,9 +21,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
-  <si>
-    <t xml:space="preserve">Name</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="11">
+  <si>
+    <t xml:space="preserve">Employee</t>
   </si>
   <si>
     <t xml:space="preserve">John</t>
@@ -32,14 +33,36 @@
   </si>
   <si>
     <t xml:space="preserve">Mr. Smith</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Date</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Customer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Description</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hours</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sarah Mitchell</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Railing</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="General"/>
+    <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
   </numFmts>
   <fonts count="6">
     <font>
@@ -122,16 +145,28 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="6">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -327,28 +362,28 @@
   <dimension ref="A1:A4"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="18.29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="19"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="21.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="18.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="19"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="21.86"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="24.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="22.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+    <row r="2" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="22.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="s">
+    <row r="3" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="3" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="22.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2" t="s">
+    <row r="4" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="3" t="s">
         <v>3</v>
       </c>
     </row>
@@ -361,4 +396,69 @@
     <oddFooter/>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="19.52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="13.39"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="11.06"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="9.71"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="0" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" s="0" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1" s="0" t="s">
+        <v>7</v>
+      </c>
+      <c r="E1" s="0" t="s">
+        <v>0</v>
+      </c>
+      <c r="F1" s="0" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="4" t="n">
+        <v>46082</v>
+      </c>
+      <c r="B2" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="F2" s="0" t="n">
+        <v>1.5</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>